<commit_message>
subir listados campaña corazul10
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_wednesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_wednesday.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/Library/Mobile Documents/com~apple~CloudDocs/GRIDDED.AGENCY/PROYECTOS/2026/02 MIRAMAR CRUISES/Agente Descubierta/03 Campañas agente descubierta/260407 Corazul/listado envios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02801222-14D6-F74C-B1D4-6556E037FBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6076B68C-408C-DE44-999C-2B33D8F20E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9180" yWindow="600" windowWidth="27240" windowHeight="20260" xr2:uid="{7F4A6893-5380-1848-9F9B-1ED428146709}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="322">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -178,9 +178,6 @@
   </si>
   <si>
     <t>ROSAGRO ESCAMEZ</t>
-  </si>
-  <si>
-    <t>677912314 - Mirna</t>
   </si>
   <si>
     <t>fmirnab@gmail.com</t>
@@ -1588,17 +1585,17 @@
       <c r="C6" t="s">
         <v>43</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6">
+        <v>677912314</v>
+      </c>
+      <c r="E6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>45</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>46</v>
-      </c>
-      <c r="G6" t="s">
-        <v>47</v>
       </c>
       <c r="H6" s="1">
         <v>45836</v>
@@ -1609,22 +1606,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>49</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>50</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>51</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>52</v>
-      </c>
-      <c r="G7" t="s">
-        <v>53</v>
       </c>
       <c r="H7" s="1">
         <v>45899</v>
@@ -1638,19 +1635,19 @@
         <v>36</v>
       </c>
       <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
         <v>54</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>55</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>56</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>57</v>
-      </c>
-      <c r="G8" t="s">
-        <v>58</v>
       </c>
       <c r="H8" s="1">
         <v>45861</v>
@@ -1661,22 +1658,22 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
         <v>59</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>60</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>61</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>62</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>63</v>
-      </c>
-      <c r="G9" t="s">
-        <v>64</v>
       </c>
       <c r="H9" s="1">
         <v>45881</v>
@@ -1687,22 +1684,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
         <v>65</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>66</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>67</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>68</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>69</v>
-      </c>
-      <c r="G10" t="s">
-        <v>70</v>
       </c>
       <c r="H10" s="1">
         <v>45914</v>
@@ -1713,22 +1710,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>72</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>73</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>74</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>75</v>
-      </c>
-      <c r="G11" t="s">
-        <v>76</v>
       </c>
       <c r="H11" s="1">
         <v>45825</v>
@@ -1739,19 +1736,19 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" t="s">
         <v>77</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>78</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>79</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>80</v>
-      </c>
-      <c r="F12" t="s">
-        <v>81</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
@@ -1765,22 +1762,22 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" t="s">
         <v>82</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>83</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>84</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>85</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>86</v>
-      </c>
-      <c r="G13" t="s">
-        <v>87</v>
       </c>
       <c r="H13" s="1">
         <v>45879</v>
@@ -1791,22 +1788,22 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" t="s">
         <v>88</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>89</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>90</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>91</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>92</v>
-      </c>
-      <c r="G14" t="s">
-        <v>93</v>
       </c>
       <c r="H14" s="1">
         <v>45904</v>
@@ -1817,22 +1814,22 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" t="s">
         <v>94</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>95</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>96</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>97</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>98</v>
-      </c>
-      <c r="G15" t="s">
-        <v>99</v>
       </c>
       <c r="H15" s="1">
         <v>45878</v>
@@ -1843,22 +1840,22 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" t="s">
         <v>100</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>101</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>102</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>103</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>104</v>
-      </c>
-      <c r="G16" t="s">
-        <v>105</v>
       </c>
       <c r="H16" s="1">
         <v>45959</v>
@@ -1869,22 +1866,22 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s">
         <v>106</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>107</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>108</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>109</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>110</v>
-      </c>
-      <c r="G17" t="s">
-        <v>111</v>
       </c>
       <c r="H17" s="1">
         <v>46019</v>
@@ -1895,22 +1892,22 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" t="s">
         <v>112</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>113</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>114</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>115</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>116</v>
-      </c>
-      <c r="G18" t="s">
-        <v>117</v>
       </c>
       <c r="H18" s="1">
         <v>45856</v>
@@ -1924,19 +1921,19 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" t="s">
         <v>118</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>119</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>120</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>121</v>
-      </c>
-      <c r="G19" t="s">
-        <v>122</v>
       </c>
       <c r="H19" s="1">
         <v>45877</v>
@@ -1947,22 +1944,22 @@
         <v>8</v>
       </c>
       <c r="B20" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" t="s">
         <v>123</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>124</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>125</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>126</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>127</v>
-      </c>
-      <c r="G20" t="s">
-        <v>128</v>
       </c>
       <c r="H20" s="1">
         <v>45858</v>
@@ -1973,22 +1970,22 @@
         <v>8</v>
       </c>
       <c r="B21" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" t="s">
         <v>129</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>130</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>131</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>132</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>133</v>
-      </c>
-      <c r="G21" t="s">
-        <v>134</v>
       </c>
       <c r="H21" s="1">
         <v>45828</v>
@@ -1999,22 +1996,22 @@
         <v>13</v>
       </c>
       <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" t="s">
         <v>135</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>136</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>137</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>138</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>139</v>
-      </c>
-      <c r="G22" t="s">
-        <v>140</v>
       </c>
       <c r="H22" s="1">
         <v>45893</v>
@@ -2025,22 +2022,22 @@
         <v>13</v>
       </c>
       <c r="B23" t="s">
+        <v>140</v>
+      </c>
+      <c r="C23" t="s">
         <v>141</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>142</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>143</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>144</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>145</v>
-      </c>
-      <c r="G23" t="s">
-        <v>146</v>
       </c>
       <c r="H23" s="1">
         <v>45919</v>
@@ -2051,22 +2048,22 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" t="s">
         <v>147</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>148</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>149</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>150</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>151</v>
-      </c>
-      <c r="G24" t="s">
-        <v>152</v>
       </c>
       <c r="H24" s="1">
         <v>45865</v>
@@ -2077,22 +2074,22 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" t="s">
         <v>153</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>154</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>155</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>156</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>157</v>
-      </c>
-      <c r="G25" t="s">
-        <v>158</v>
       </c>
       <c r="H25" s="1">
         <v>45901</v>
@@ -2106,19 +2103,19 @@
         <v>14</v>
       </c>
       <c r="C26" t="s">
+        <v>158</v>
+      </c>
+      <c r="D26" t="s">
         <v>159</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>160</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>161</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>162</v>
-      </c>
-      <c r="G26" t="s">
-        <v>163</v>
       </c>
       <c r="H26" s="1">
         <v>45873</v>
@@ -2129,22 +2126,22 @@
         <v>8</v>
       </c>
       <c r="B27" t="s">
+        <v>163</v>
+      </c>
+      <c r="C27" t="s">
         <v>164</v>
-      </c>
-      <c r="C27" t="s">
-        <v>165</v>
       </c>
       <c r="D27">
         <v>605060036</v>
       </c>
       <c r="E27" t="s">
+        <v>165</v>
+      </c>
+      <c r="F27" t="s">
         <v>166</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>167</v>
-      </c>
-      <c r="G27" t="s">
-        <v>168</v>
       </c>
       <c r="H27" s="1">
         <v>45886</v>
@@ -2155,22 +2152,22 @@
         <v>8</v>
       </c>
       <c r="B28" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" t="s">
         <v>169</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>170</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>171</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>172</v>
       </c>
-      <c r="F28" t="s">
-        <v>173</v>
-      </c>
       <c r="G28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H28" s="1">
         <v>45900</v>
@@ -2181,22 +2178,22 @@
         <v>9</v>
       </c>
       <c r="B29" t="s">
+        <v>173</v>
+      </c>
+      <c r="C29" t="s">
         <v>174</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>175</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>176</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>177</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>178</v>
-      </c>
-      <c r="G29" t="s">
-        <v>179</v>
       </c>
       <c r="H29" s="1">
         <v>45867</v>
@@ -2207,19 +2204,19 @@
         <v>8</v>
       </c>
       <c r="B30" t="s">
+        <v>179</v>
+      </c>
+      <c r="C30" t="s">
         <v>180</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>181</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>182</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>183</v>
-      </c>
-      <c r="F30" t="s">
-        <v>184</v>
       </c>
       <c r="G30" t="s">
         <v>10</v>
@@ -2233,22 +2230,22 @@
         <v>11</v>
       </c>
       <c r="B31" t="s">
+        <v>184</v>
+      </c>
+      <c r="C31" t="s">
         <v>185</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>186</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>187</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>188</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>189</v>
-      </c>
-      <c r="G31" t="s">
-        <v>190</v>
       </c>
       <c r="H31" s="1">
         <v>45991</v>
@@ -2259,22 +2256,22 @@
         <v>8</v>
       </c>
       <c r="B32" t="s">
+        <v>190</v>
+      </c>
+      <c r="C32" t="s">
         <v>191</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>192</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>193</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>194</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>195</v>
-      </c>
-      <c r="G32" t="s">
-        <v>196</v>
       </c>
       <c r="H32" s="1">
         <v>45878</v>
@@ -2285,22 +2282,22 @@
         <v>8</v>
       </c>
       <c r="B33" t="s">
+        <v>196</v>
+      </c>
+      <c r="C33" t="s">
         <v>197</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>198</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>199</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>200</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>201</v>
-      </c>
-      <c r="G33" t="s">
-        <v>202</v>
       </c>
       <c r="H33" s="1">
         <v>45865</v>
@@ -2311,22 +2308,22 @@
         <v>13</v>
       </c>
       <c r="B34" t="s">
+        <v>202</v>
+      </c>
+      <c r="C34" t="s">
         <v>203</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>204</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>205</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>206</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>207</v>
-      </c>
-      <c r="G34" t="s">
-        <v>208</v>
       </c>
       <c r="H34" s="1">
         <v>45888</v>
@@ -2337,22 +2334,22 @@
         <v>9</v>
       </c>
       <c r="B35" t="s">
+        <v>208</v>
+      </c>
+      <c r="C35" t="s">
         <v>209</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>210</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>211</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>212</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>213</v>
-      </c>
-      <c r="G35" t="s">
-        <v>214</v>
       </c>
       <c r="H35" s="1">
         <v>45975</v>
@@ -2363,22 +2360,22 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
+        <v>214</v>
+      </c>
+      <c r="C36" t="s">
         <v>215</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>216</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>217</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>218</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>219</v>
-      </c>
-      <c r="G36" t="s">
-        <v>220</v>
       </c>
       <c r="H36" s="1">
         <v>45872</v>
@@ -2389,22 +2386,22 @@
         <v>8</v>
       </c>
       <c r="B37" t="s">
+        <v>220</v>
+      </c>
+      <c r="C37" t="s">
         <v>221</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>222</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>223</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>224</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>225</v>
-      </c>
-      <c r="G37" t="s">
-        <v>226</v>
       </c>
       <c r="H37" s="1">
         <v>45893</v>
@@ -2415,19 +2412,19 @@
         <v>8</v>
       </c>
       <c r="B38" t="s">
+        <v>226</v>
+      </c>
+      <c r="C38" t="s">
         <v>227</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>228</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>229</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>230</v>
-      </c>
-      <c r="F38" t="s">
-        <v>231</v>
       </c>
       <c r="G38" t="s">
         <v>18</v>
@@ -2444,19 +2441,19 @@
         <v>19</v>
       </c>
       <c r="C39" t="s">
+        <v>231</v>
+      </c>
+      <c r="D39" t="s">
         <v>232</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>233</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
         <v>234</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>235</v>
-      </c>
-      <c r="G39" t="s">
-        <v>236</v>
       </c>
       <c r="H39" s="1">
         <v>45880</v>
@@ -2467,19 +2464,19 @@
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C40" t="s">
+        <v>236</v>
+      </c>
+      <c r="D40" t="s">
         <v>237</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>238</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>239</v>
-      </c>
-      <c r="F40" t="s">
-        <v>240</v>
       </c>
       <c r="G40" t="s">
         <v>16</v>
@@ -2496,19 +2493,19 @@
         <v>12</v>
       </c>
       <c r="C41" t="s">
+        <v>240</v>
+      </c>
+      <c r="D41" t="s">
         <v>241</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>242</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>243</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>244</v>
-      </c>
-      <c r="G41" t="s">
-        <v>245</v>
       </c>
       <c r="H41" s="1">
         <v>45870</v>
@@ -2519,22 +2516,22 @@
         <v>8</v>
       </c>
       <c r="B42" t="s">
+        <v>245</v>
+      </c>
+      <c r="C42" t="s">
         <v>246</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>247</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>248</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>249</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>250</v>
-      </c>
-      <c r="G42" t="s">
-        <v>251</v>
       </c>
       <c r="H42" s="1">
         <v>45879</v>
@@ -2545,22 +2542,22 @@
         <v>8</v>
       </c>
       <c r="B43" t="s">
+        <v>251</v>
+      </c>
+      <c r="C43" t="s">
         <v>252</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>253</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>254</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>255</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>256</v>
-      </c>
-      <c r="G43" t="s">
-        <v>257</v>
       </c>
       <c r="H43" s="1">
         <v>45900</v>
@@ -2571,22 +2568,22 @@
         <v>13</v>
       </c>
       <c r="B44" t="s">
+        <v>257</v>
+      </c>
+      <c r="C44" t="s">
         <v>258</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>259</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>260</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>261</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>262</v>
-      </c>
-      <c r="G44" t="s">
-        <v>263</v>
       </c>
       <c r="H44" s="1">
         <v>45941</v>
@@ -2597,22 +2594,22 @@
         <v>8</v>
       </c>
       <c r="B45" t="s">
+        <v>263</v>
+      </c>
+      <c r="C45" t="s">
         <v>264</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>265</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>266</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>267</v>
       </c>
-      <c r="F45" t="s">
-        <v>268</v>
-      </c>
       <c r="G45" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H45" s="1">
         <v>45893</v>
@@ -2623,22 +2620,22 @@
         <v>8</v>
       </c>
       <c r="B46" t="s">
+        <v>268</v>
+      </c>
+      <c r="C46" t="s">
         <v>269</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>270</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>271</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>272</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>273</v>
-      </c>
-      <c r="G46" t="s">
-        <v>274</v>
       </c>
       <c r="H46" s="1">
         <v>45976</v>
@@ -2649,19 +2646,19 @@
         <v>9</v>
       </c>
       <c r="B47" t="s">
+        <v>274</v>
+      </c>
+      <c r="C47" t="s">
         <v>275</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>276</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>277</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>278</v>
-      </c>
-      <c r="F47" t="s">
-        <v>279</v>
       </c>
       <c r="G47" t="s">
         <v>16</v>
@@ -2675,22 +2672,22 @@
         <v>8</v>
       </c>
       <c r="B48" t="s">
+        <v>279</v>
+      </c>
+      <c r="C48" t="s">
         <v>280</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>281</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>282</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>283</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>284</v>
-      </c>
-      <c r="G48" t="s">
-        <v>285</v>
       </c>
       <c r="H48" s="1">
         <v>45988</v>
@@ -2701,22 +2698,22 @@
         <v>8</v>
       </c>
       <c r="B49" t="s">
+        <v>285</v>
+      </c>
+      <c r="C49" t="s">
         <v>286</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>287</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>288</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
         <v>289</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>290</v>
-      </c>
-      <c r="G49" t="s">
-        <v>291</v>
       </c>
       <c r="H49" s="1">
         <v>45988</v>
@@ -2727,22 +2724,22 @@
         <v>9</v>
       </c>
       <c r="B50" t="s">
+        <v>291</v>
+      </c>
+      <c r="C50" t="s">
         <v>292</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>293</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>294</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>295</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>296</v>
-      </c>
-      <c r="G50" t="s">
-        <v>297</v>
       </c>
       <c r="H50" s="1">
         <v>45975</v>
@@ -2753,22 +2750,22 @@
         <v>8</v>
       </c>
       <c r="B51" t="s">
+        <v>297</v>
+      </c>
+      <c r="C51" t="s">
         <v>298</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>299</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>300</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
         <v>301</v>
       </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>302</v>
-      </c>
-      <c r="G51" t="s">
-        <v>303</v>
       </c>
       <c r="H51" s="1">
         <v>45988</v>
@@ -2776,25 +2773,25 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>303</v>
+      </c>
+      <c r="B52" t="s">
         <v>304</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>305</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>306</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>307</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>308</v>
       </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>309</v>
-      </c>
-      <c r="G52" t="s">
-        <v>310</v>
       </c>
       <c r="H52" s="1">
         <v>46011</v>
@@ -2805,22 +2802,22 @@
         <v>8</v>
       </c>
       <c r="B53" t="s">
+        <v>310</v>
+      </c>
+      <c r="C53" t="s">
         <v>311</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>312</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>313</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>314</v>
       </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
         <v>315</v>
-      </c>
-      <c r="G53" t="s">
-        <v>316</v>
       </c>
       <c r="H53" s="1">
         <v>45998</v>
@@ -2831,22 +2828,22 @@
         <v>8</v>
       </c>
       <c r="B54" t="s">
+        <v>316</v>
+      </c>
+      <c r="C54" t="s">
         <v>317</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>318</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>319</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>320</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>321</v>
-      </c>
-      <c r="G54" t="s">
-        <v>322</v>
       </c>
       <c r="H54" s="1">
         <v>46019</v>

</xml_diff>

<commit_message>
subir listados campaña corazul2.1
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_wednesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_wednesday.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6076B68C-408C-DE44-999C-2B33D8F20E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A479F7-119D-AF41-B5E1-D66A3208DB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9180" yWindow="600" windowWidth="27240" windowHeight="20260" xr2:uid="{7F4A6893-5380-1848-9F9B-1ED428146709}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$54</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$52</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="310">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -93,9 +93,6 @@
     <t>BEATRIZ</t>
   </si>
   <si>
-    <t>MARIA</t>
-  </si>
-  <si>
     <t>GRANADA</t>
   </si>
   <si>
@@ -106,39 +103,6 @@
   </si>
   <si>
     <t>PAULA</t>
-  </si>
-  <si>
-    <t>Joan Miquel</t>
-  </si>
-  <si>
-    <t>Forteza Fuster</t>
-  </si>
-  <si>
-    <t>685530021</t>
-  </si>
-  <si>
-    <t>luciagonzalez199985@gmail.com</t>
-  </si>
-  <si>
-    <t>Calle Can Catlari 54, bajos A</t>
-  </si>
-  <si>
-    <t>Pla de na Tesa, Marratxi</t>
-  </si>
-  <si>
-    <t>SOSA FERNANDEZ</t>
-  </si>
-  <si>
-    <t>722234610</t>
-  </si>
-  <si>
-    <t>mariasosafernandez14@gmail.com</t>
-  </si>
-  <si>
-    <t>CALLE MONTEALTO I, 7</t>
-  </si>
-  <si>
-    <t>CALLES</t>
   </si>
   <si>
     <t>Miguel</t>
@@ -1117,8 +1081,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F484A26-905F-264F-B00B-DD3436D50B8F}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H54" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H54" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F484A26-905F-264F-B00B-DD3436D50B8F}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H52" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H52" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{8421434A-6D24-CA47-8CF1-023952E0C6FA}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{9F8BCCDB-15E3-1F4F-8141-86D49716F498}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1430,7 +1394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28AF013B-1C7E-974D-BCF6-767DBC07596A}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1473,132 +1437,132 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2">
+        <v>627625508</v>
+      </c>
+      <c r="E2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>23</v>
       </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
       <c r="H2" s="1">
-        <v>45814</v>
+        <v>45964</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>28</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>29</v>
       </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
       <c r="H3" s="1">
-        <v>45855</v>
+        <v>45809</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4">
+        <v>677912314</v>
+      </c>
+      <c r="E4" t="s">
         <v>32</v>
       </c>
-      <c r="D4">
-        <v>627625508</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>33</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>34</v>
       </c>
-      <c r="G4" t="s">
-        <v>35</v>
-      </c>
       <c r="H4" s="1">
-        <v>45964</v>
+        <v>45836</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>37</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>39</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>40</v>
       </c>
-      <c r="G5" t="s">
-        <v>41</v>
-      </c>
       <c r="H5" s="1">
-        <v>45809</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
         <v>42</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>43</v>
       </c>
-      <c r="D6">
-        <v>677912314</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>44</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" t="s">
-        <v>46</v>
-      </c>
       <c r="H6" s="1">
-        <v>45836</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1606,33 +1570,33 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>48</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>49</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="G7" t="s">
-        <v>52</v>
-      </c>
       <c r="H7" s="1">
-        <v>45899</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
         <v>53</v>
@@ -1650,7 +1614,7 @@
         <v>57</v>
       </c>
       <c r="H8" s="1">
-        <v>45861</v>
+        <v>45914</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1676,12 +1640,12 @@
         <v>63</v>
       </c>
       <c r="H9" s="1">
-        <v>45881</v>
+        <v>45825</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>64</v>
@@ -1699,36 +1663,36 @@
         <v>68</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="H10" s="1">
-        <v>45914</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>71</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>72</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>73</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>74</v>
       </c>
-      <c r="G11" t="s">
-        <v>75</v>
-      </c>
       <c r="H11" s="1">
-        <v>45825</v>
+        <v>45879</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1736,30 +1700,30 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" t="s">
         <v>76</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>77</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>78</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>80</v>
       </c>
-      <c r="G12" t="s">
-        <v>18</v>
-      </c>
       <c r="H12" s="1">
-        <v>45876</v>
+        <v>45904</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
         <v>81</v>
@@ -1780,12 +1744,12 @@
         <v>86</v>
       </c>
       <c r="H13" s="1">
-        <v>45879</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
         <v>87</v>
@@ -1806,7 +1770,7 @@
         <v>92</v>
       </c>
       <c r="H14" s="1">
-        <v>45904</v>
+        <v>45959</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -1832,12 +1796,12 @@
         <v>98</v>
       </c>
       <c r="H15" s="1">
-        <v>45878</v>
+        <v>46019</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
         <v>99</v>
@@ -1858,59 +1822,59 @@
         <v>104</v>
       </c>
       <c r="H16" s="1">
-        <v>45959</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
         <v>105</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>106</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>107</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>108</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>109</v>
       </c>
-      <c r="G17" t="s">
-        <v>110</v>
-      </c>
       <c r="H17" s="1">
-        <v>46019</v>
+        <v>45877</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" t="s">
         <v>111</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>112</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>113</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>114</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>115</v>
       </c>
-      <c r="G18" t="s">
-        <v>116</v>
-      </c>
       <c r="H18" s="1">
-        <v>45856</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1918,7 +1882,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
         <v>117</v>
@@ -1936,12 +1900,12 @@
         <v>121</v>
       </c>
       <c r="H19" s="1">
-        <v>45877</v>
+        <v>45828</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
         <v>122</v>
@@ -1962,12 +1926,12 @@
         <v>127</v>
       </c>
       <c r="H20" s="1">
-        <v>45858</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
         <v>128</v>
@@ -1988,12 +1952,12 @@
         <v>133</v>
       </c>
       <c r="H21" s="1">
-        <v>45828</v>
+        <v>45919</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B22" t="s">
         <v>134</v>
@@ -2014,12 +1978,12 @@
         <v>139</v>
       </c>
       <c r="H22" s="1">
-        <v>45893</v>
+        <v>45865</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
         <v>140</v>
@@ -2040,7 +2004,7 @@
         <v>145</v>
       </c>
       <c r="H23" s="1">
-        <v>45919</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -2048,25 +2012,25 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" t="s">
         <v>146</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>147</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>148</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>149</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>150</v>
       </c>
-      <c r="G24" t="s">
-        <v>151</v>
-      </c>
       <c r="H24" s="1">
-        <v>45865</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -2074,25 +2038,25 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
+        <v>151</v>
+      </c>
+      <c r="C25" t="s">
         <v>152</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25">
+        <v>605060036</v>
+      </c>
+      <c r="E25" t="s">
         <v>153</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
         <v>154</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>155</v>
       </c>
-      <c r="F25" t="s">
-        <v>156</v>
-      </c>
-      <c r="G25" t="s">
-        <v>157</v>
-      </c>
       <c r="H25" s="1">
-        <v>45901</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -2100,51 +2064,51 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>156</v>
       </c>
       <c r="C26" t="s">
+        <v>157</v>
+      </c>
+      <c r="D26" t="s">
         <v>158</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>159</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>160</v>
       </c>
-      <c r="F26" t="s">
-        <v>161</v>
-      </c>
       <c r="G26" t="s">
-        <v>162</v>
+        <v>121</v>
       </c>
       <c r="H26" s="1">
-        <v>45873</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
+        <v>161</v>
+      </c>
+      <c r="C27" t="s">
+        <v>162</v>
+      </c>
+      <c r="D27" t="s">
         <v>163</v>
       </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
         <v>164</v>
       </c>
-      <c r="D27">
-        <v>605060036</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>165</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>166</v>
       </c>
-      <c r="G27" t="s">
-        <v>167</v>
-      </c>
       <c r="H27" s="1">
-        <v>45886</v>
+        <v>45867</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -2152,51 +2116,51 @@
         <v>8</v>
       </c>
       <c r="B28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C28" t="s">
         <v>168</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>169</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>170</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>171</v>
       </c>
-      <c r="F28" t="s">
-        <v>172</v>
-      </c>
       <c r="G28" t="s">
-        <v>133</v>
+        <v>10</v>
       </c>
       <c r="H28" s="1">
-        <v>45900</v>
+        <v>45879</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B29" t="s">
+        <v>172</v>
+      </c>
+      <c r="C29" t="s">
         <v>173</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>174</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>175</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>176</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>177</v>
       </c>
-      <c r="G29" t="s">
-        <v>178</v>
-      </c>
       <c r="H29" s="1">
-        <v>45867</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -2204,30 +2168,30 @@
         <v>8</v>
       </c>
       <c r="B30" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" t="s">
         <v>179</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>180</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>181</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>182</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>183</v>
       </c>
-      <c r="G30" t="s">
-        <v>10</v>
-      </c>
       <c r="H30" s="1">
-        <v>45879</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
         <v>184</v>
@@ -2248,12 +2212,12 @@
         <v>189</v>
       </c>
       <c r="H31" s="1">
-        <v>45991</v>
+        <v>45865</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
         <v>190</v>
@@ -2274,12 +2238,12 @@
         <v>195</v>
       </c>
       <c r="H32" s="1">
-        <v>45878</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
         <v>196</v>
@@ -2300,12 +2264,12 @@
         <v>201</v>
       </c>
       <c r="H33" s="1">
-        <v>45865</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
         <v>202</v>
@@ -2326,12 +2290,12 @@
         <v>207</v>
       </c>
       <c r="H34" s="1">
-        <v>45888</v>
+        <v>45872</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
         <v>208</v>
@@ -2352,7 +2316,7 @@
         <v>213</v>
       </c>
       <c r="H35" s="1">
-        <v>45975</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -2375,10 +2339,10 @@
         <v>218</v>
       </c>
       <c r="G36" t="s">
-        <v>219</v>
+        <v>17</v>
       </c>
       <c r="H36" s="1">
-        <v>45872</v>
+        <v>45936</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -2386,51 +2350,51 @@
         <v>8</v>
       </c>
       <c r="B37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>219</v>
+      </c>
+      <c r="D37" t="s">
         <v>220</v>
       </c>
-      <c r="C37" t="s">
+      <c r="E37" t="s">
         <v>221</v>
       </c>
-      <c r="D37" t="s">
+      <c r="F37" t="s">
         <v>222</v>
       </c>
-      <c r="E37" t="s">
+      <c r="G37" t="s">
         <v>223</v>
       </c>
-      <c r="F37" t="s">
-        <v>224</v>
-      </c>
-      <c r="G37" t="s">
-        <v>225</v>
-      </c>
       <c r="H37" s="1">
-        <v>45893</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" t="s">
+        <v>224</v>
+      </c>
+      <c r="D38" t="s">
+        <v>225</v>
+      </c>
+      <c r="E38" t="s">
         <v>226</v>
       </c>
-      <c r="C38" t="s">
+      <c r="F38" t="s">
         <v>227</v>
       </c>
-      <c r="D38" t="s">
-        <v>228</v>
-      </c>
-      <c r="E38" t="s">
-        <v>229</v>
-      </c>
-      <c r="F38" t="s">
-        <v>230</v>
-      </c>
       <c r="G38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H38" s="1">
-        <v>45936</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -2438,51 +2402,51 @@
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C39" t="s">
+        <v>228</v>
+      </c>
+      <c r="D39" t="s">
+        <v>229</v>
+      </c>
+      <c r="E39" t="s">
+        <v>230</v>
+      </c>
+      <c r="F39" t="s">
         <v>231</v>
       </c>
-      <c r="D39" t="s">
+      <c r="G39" t="s">
         <v>232</v>
       </c>
-      <c r="E39" t="s">
-        <v>233</v>
-      </c>
-      <c r="F39" t="s">
-        <v>234</v>
-      </c>
-      <c r="G39" t="s">
-        <v>235</v>
-      </c>
       <c r="H39" s="1">
-        <v>45880</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>233</v>
       </c>
       <c r="C40" t="s">
+        <v>234</v>
+      </c>
+      <c r="D40" t="s">
+        <v>235</v>
+      </c>
+      <c r="E40" t="s">
         <v>236</v>
       </c>
-      <c r="D40" t="s">
+      <c r="F40" t="s">
         <v>237</v>
       </c>
-      <c r="E40" t="s">
+      <c r="G40" t="s">
         <v>238</v>
       </c>
-      <c r="F40" t="s">
-        <v>239</v>
-      </c>
-      <c r="G40" t="s">
-        <v>16</v>
-      </c>
       <c r="H40" s="1">
-        <v>45900</v>
+        <v>45879</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -2490,7 +2454,7 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>239</v>
       </c>
       <c r="C41" t="s">
         <v>240</v>
@@ -2508,12 +2472,12 @@
         <v>244</v>
       </c>
       <c r="H41" s="1">
-        <v>45870</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
         <v>245</v>
@@ -2534,7 +2498,7 @@
         <v>250</v>
       </c>
       <c r="H42" s="1">
-        <v>45879</v>
+        <v>45941</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2557,62 +2521,62 @@
         <v>255</v>
       </c>
       <c r="G43" t="s">
-        <v>256</v>
+        <v>145</v>
       </c>
       <c r="H43" s="1">
-        <v>45900</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
+        <v>256</v>
+      </c>
+      <c r="C44" t="s">
         <v>257</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>258</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>259</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>260</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>261</v>
       </c>
-      <c r="G44" t="s">
-        <v>262</v>
-      </c>
       <c r="H44" s="1">
-        <v>45941</v>
+        <v>45976</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B45" t="s">
+        <v>262</v>
+      </c>
+      <c r="C45" t="s">
         <v>263</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>264</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>265</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>266</v>
       </c>
-      <c r="F45" t="s">
-        <v>267</v>
-      </c>
       <c r="G45" t="s">
-        <v>157</v>
+        <v>15</v>
       </c>
       <c r="H45" s="1">
-        <v>45893</v>
+        <v>45911</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2620,56 +2584,56 @@
         <v>8</v>
       </c>
       <c r="B46" t="s">
+        <v>267</v>
+      </c>
+      <c r="C46" t="s">
         <v>268</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>269</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>270</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>271</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>272</v>
       </c>
-      <c r="G46" t="s">
-        <v>273</v>
-      </c>
       <c r="H46" s="1">
-        <v>45976</v>
+        <v>45988</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
+        <v>273</v>
+      </c>
+      <c r="C47" t="s">
         <v>274</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>275</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>276</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>277</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>278</v>
       </c>
-      <c r="G47" t="s">
-        <v>16</v>
-      </c>
       <c r="H47" s="1">
-        <v>45911</v>
+        <v>45988</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B48" t="s">
         <v>279</v>
@@ -2690,7 +2654,7 @@
         <v>284</v>
       </c>
       <c r="H48" s="1">
-        <v>45988</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -2721,28 +2685,28 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>291</v>
       </c>
       <c r="B50" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D50" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E50" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F50" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G50" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H50" s="1">
-        <v>45975</v>
+        <v>46011</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
@@ -2750,30 +2714,30 @@
         <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C51" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D51" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E51" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F51" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G51" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H51" s="1">
-        <v>45988</v>
+        <v>45998</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>303</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
         <v>304</v>
@@ -2794,58 +2758,6 @@
         <v>309</v>
       </c>
       <c r="H52" s="1">
-        <v>46011</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>8</v>
-      </c>
-      <c r="B53" t="s">
-        <v>310</v>
-      </c>
-      <c r="C53" t="s">
-        <v>311</v>
-      </c>
-      <c r="D53" t="s">
-        <v>312</v>
-      </c>
-      <c r="E53" t="s">
-        <v>313</v>
-      </c>
-      <c r="F53" t="s">
-        <v>314</v>
-      </c>
-      <c r="G53" t="s">
-        <v>315</v>
-      </c>
-      <c r="H53" s="1">
-        <v>45998</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>8</v>
-      </c>
-      <c r="B54" t="s">
-        <v>316</v>
-      </c>
-      <c r="C54" t="s">
-        <v>317</v>
-      </c>
-      <c r="D54" t="s">
-        <v>318</v>
-      </c>
-      <c r="E54" t="s">
-        <v>319</v>
-      </c>
-      <c r="F54" t="s">
-        <v>320</v>
-      </c>
-      <c r="G54" t="s">
-        <v>321</v>
-      </c>
-      <c r="H54" s="1">
         <v>46019</v>
       </c>
     </row>

</xml_diff>

<commit_message>
subir listados campaña corazul2.2
</commit_message>
<xml_diff>
--- a/campanas/260413_corazul/corazul_1_wednesday.xlsx
+++ b/campanas/260413_corazul/corazul_1_wednesday.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegopaezmacias/GRIDDED.AGENCY local/00_GRIDDED AGENCY/cdn/campanas/260413_corazul/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A479F7-119D-AF41-B5E1-D66A3208DB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9617C374-448E-D34E-99FD-F173621FC879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9180" yWindow="600" windowWidth="27240" windowHeight="20260" xr2:uid="{7F4A6893-5380-1848-9F9B-1ED428146709}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="campaña 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$52</definedName>
+    <definedName name="DatosExternos_2" localSheetId="0" hidden="1">'campaña 1'!$A$1:$H$51</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="304">
   <si>
     <t>nombreNaviera</t>
   </si>
@@ -307,24 +307,6 @@
   </si>
   <si>
     <t>Punta Umbria</t>
-  </si>
-  <si>
-    <t>TRESSY</t>
-  </si>
-  <si>
-    <t>COYERE</t>
-  </si>
-  <si>
-    <t>0641244256</t>
-  </si>
-  <si>
-    <t>kenarudy3@gmail.com</t>
-  </si>
-  <si>
-    <t>3 ALLEE JEAN LEON JEROME</t>
-  </si>
-  <si>
-    <t>VALENTINI</t>
   </si>
   <si>
     <t>MIGUEL ANGEL</t>
@@ -1081,8 +1063,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F484A26-905F-264F-B00B-DD3436D50B8F}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H52" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:H52" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F484A26-905F-264F-B00B-DD3436D50B8F}" name="Ventas_Cuadruples_2025" displayName="Ventas_Cuadruples_2025" ref="A1:H51" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H51" xr:uid="{7B6879F4-F5E9-40D9-A981-23B705F0A713}"/>
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{8421434A-6D24-CA47-8CF1-023952E0C6FA}" uniqueName="2" name="nombreNaviera" queryTableFieldId="2" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{9F8BCCDB-15E3-1F4F-8141-86D49716F498}" uniqueName="3" name="nombreCliente" queryTableFieldId="3" dataDxfId="6"/>
@@ -1394,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28AF013B-1C7E-974D-BCF6-767DBC07596A}">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -1749,7 +1731,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>87</v>
@@ -1770,7 +1752,7 @@
         <v>92</v>
       </c>
       <c r="H14" s="1">
-        <v>45959</v>
+        <v>46019</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -1796,33 +1778,33 @@
         <v>98</v>
       </c>
       <c r="H15" s="1">
-        <v>46019</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
         <v>99</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>100</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>101</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>102</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>103</v>
       </c>
-      <c r="G16" t="s">
-        <v>104</v>
-      </c>
       <c r="H16" s="1">
-        <v>45856</v>
+        <v>45877</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -1830,7 +1812,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
         <v>105</v>
@@ -1848,7 +1830,7 @@
         <v>109</v>
       </c>
       <c r="H17" s="1">
-        <v>45877</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -1874,12 +1856,12 @@
         <v>115</v>
       </c>
       <c r="H18" s="1">
-        <v>45858</v>
+        <v>45828</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
         <v>116</v>
@@ -1900,7 +1882,7 @@
         <v>121</v>
       </c>
       <c r="H19" s="1">
-        <v>45828</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -1926,12 +1908,12 @@
         <v>127</v>
       </c>
       <c r="H20" s="1">
-        <v>45893</v>
+        <v>45919</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
         <v>128</v>
@@ -1952,7 +1934,7 @@
         <v>133</v>
       </c>
       <c r="H21" s="1">
-        <v>45919</v>
+        <v>45865</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -1978,7 +1960,7 @@
         <v>139</v>
       </c>
       <c r="H22" s="1">
-        <v>45865</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1986,25 +1968,25 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" t="s">
         <v>140</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>141</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>142</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>143</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>144</v>
       </c>
-      <c r="G23" t="s">
-        <v>145</v>
-      </c>
       <c r="H23" s="1">
-        <v>45901</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -2012,25 +1994,25 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="C24" t="s">
         <v>146</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24">
+        <v>605060036</v>
+      </c>
+      <c r="E24" t="s">
         <v>147</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>148</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>149</v>
       </c>
-      <c r="G24" t="s">
-        <v>150</v>
-      </c>
       <c r="H24" s="1">
-        <v>45873</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -2038,13 +2020,13 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" t="s">
         <v>151</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>152</v>
-      </c>
-      <c r="D25">
-        <v>605060036</v>
       </c>
       <c r="E25" t="s">
         <v>153</v>
@@ -2053,41 +2035,41 @@
         <v>154</v>
       </c>
       <c r="G25" t="s">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="H25" s="1">
-        <v>45886</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C26" t="s">
         <v>156</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>157</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>158</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>159</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>160</v>
       </c>
-      <c r="G26" t="s">
-        <v>121</v>
-      </c>
       <c r="H26" s="1">
-        <v>45900</v>
+        <v>45867</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
         <v>161</v>
@@ -2105,41 +2087,41 @@
         <v>165</v>
       </c>
       <c r="G27" t="s">
-        <v>166</v>
+        <v>10</v>
       </c>
       <c r="H27" s="1">
-        <v>45867</v>
+        <v>45879</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
+        <v>166</v>
+      </c>
+      <c r="C28" t="s">
         <v>167</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>168</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>169</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>170</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>171</v>
       </c>
-      <c r="G28" t="s">
-        <v>10</v>
-      </c>
       <c r="H28" s="1">
-        <v>45879</v>
+        <v>45991</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>172</v>
@@ -2160,7 +2142,7 @@
         <v>177</v>
       </c>
       <c r="H29" s="1">
-        <v>45991</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -2186,12 +2168,12 @@
         <v>183</v>
       </c>
       <c r="H30" s="1">
-        <v>45878</v>
+        <v>45865</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
         <v>184</v>
@@ -2212,12 +2194,12 @@
         <v>189</v>
       </c>
       <c r="H31" s="1">
-        <v>45865</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B32" t="s">
         <v>190</v>
@@ -2238,12 +2220,12 @@
         <v>195</v>
       </c>
       <c r="H32" s="1">
-        <v>45888</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B33" t="s">
         <v>196</v>
@@ -2264,7 +2246,7 @@
         <v>201</v>
       </c>
       <c r="H33" s="1">
-        <v>45975</v>
+        <v>45872</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -2290,7 +2272,7 @@
         <v>207</v>
       </c>
       <c r="H34" s="1">
-        <v>45872</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -2313,10 +2295,10 @@
         <v>212</v>
       </c>
       <c r="G35" t="s">
-        <v>213</v>
+        <v>17</v>
       </c>
       <c r="H35" s="1">
-        <v>45893</v>
+        <v>45936</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -2324,77 +2306,77 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" t="s">
+        <v>213</v>
+      </c>
+      <c r="D36" t="s">
         <v>214</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" t="s">
         <v>215</v>
       </c>
-      <c r="D36" t="s">
+      <c r="F36" t="s">
         <v>216</v>
       </c>
-      <c r="E36" t="s">
+      <c r="G36" t="s">
         <v>217</v>
       </c>
-      <c r="F36" t="s">
-        <v>218</v>
-      </c>
-      <c r="G36" t="s">
-        <v>17</v>
-      </c>
       <c r="H36" s="1">
-        <v>45936</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s">
+        <v>218</v>
+      </c>
+      <c r="D37" t="s">
         <v>219</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>220</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>221</v>
       </c>
-      <c r="F37" t="s">
-        <v>222</v>
-      </c>
       <c r="G37" t="s">
-        <v>223</v>
+        <v>15</v>
       </c>
       <c r="H37" s="1">
-        <v>45880</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="C38" t="s">
+        <v>222</v>
+      </c>
+      <c r="D38" t="s">
+        <v>223</v>
+      </c>
+      <c r="E38" t="s">
         <v>224</v>
       </c>
-      <c r="D38" t="s">
+      <c r="F38" t="s">
         <v>225</v>
       </c>
-      <c r="E38" t="s">
+      <c r="G38" t="s">
         <v>226</v>
       </c>
-      <c r="F38" t="s">
-        <v>227</v>
-      </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
       <c r="H38" s="1">
-        <v>45900</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -2402,7 +2384,7 @@
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>227</v>
       </c>
       <c r="C39" t="s">
         <v>228</v>
@@ -2420,7 +2402,7 @@
         <v>232</v>
       </c>
       <c r="H39" s="1">
-        <v>45870</v>
+        <v>45879</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2446,12 +2428,12 @@
         <v>238</v>
       </c>
       <c r="H40" s="1">
-        <v>45879</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
         <v>239</v>
@@ -2472,12 +2454,12 @@
         <v>244</v>
       </c>
       <c r="H41" s="1">
-        <v>45900</v>
+        <v>45941</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B42" t="s">
         <v>245</v>
@@ -2495,10 +2477,10 @@
         <v>249</v>
       </c>
       <c r="G42" t="s">
-        <v>250</v>
+        <v>139</v>
       </c>
       <c r="H42" s="1">
-        <v>45941</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2506,30 +2488,30 @@
         <v>8</v>
       </c>
       <c r="B43" t="s">
+        <v>250</v>
+      </c>
+      <c r="C43" t="s">
         <v>251</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>252</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>253</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>254</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>255</v>
       </c>
-      <c r="G43" t="s">
-        <v>145</v>
-      </c>
       <c r="H43" s="1">
-        <v>45893</v>
+        <v>45976</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B44" t="s">
         <v>256</v>
@@ -2547,36 +2529,36 @@
         <v>260</v>
       </c>
       <c r="G44" t="s">
-        <v>261</v>
+        <v>15</v>
       </c>
       <c r="H44" s="1">
-        <v>45976</v>
+        <v>45911</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
+        <v>261</v>
+      </c>
+      <c r="C45" t="s">
         <v>262</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>263</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>264</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>265</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>266</v>
       </c>
-      <c r="G45" t="s">
-        <v>15</v>
-      </c>
       <c r="H45" s="1">
-        <v>45911</v>
+        <v>45988</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2607,7 +2589,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B47" t="s">
         <v>273</v>
@@ -2628,12 +2610,12 @@
         <v>278</v>
       </c>
       <c r="H47" s="1">
-        <v>45988</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
         <v>279</v>
@@ -2654,38 +2636,38 @@
         <v>284</v>
       </c>
       <c r="H48" s="1">
-        <v>45975</v>
+        <v>45988</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>8</v>
+        <v>285</v>
       </c>
       <c r="B49" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C49" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D49" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E49" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F49" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G49" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H49" s="1">
-        <v>45988</v>
+        <v>46011</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>291</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
         <v>292</v>
@@ -2706,7 +2688,7 @@
         <v>297</v>
       </c>
       <c r="H50" s="1">
-        <v>46011</v>
+        <v>45998</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
@@ -2732,32 +2714,6 @@
         <v>303</v>
       </c>
       <c r="H51" s="1">
-        <v>45998</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>8</v>
-      </c>
-      <c r="B52" t="s">
-        <v>304</v>
-      </c>
-      <c r="C52" t="s">
-        <v>305</v>
-      </c>
-      <c r="D52" t="s">
-        <v>306</v>
-      </c>
-      <c r="E52" t="s">
-        <v>307</v>
-      </c>
-      <c r="F52" t="s">
-        <v>308</v>
-      </c>
-      <c r="G52" t="s">
-        <v>309</v>
-      </c>
-      <c r="H52" s="1">
         <v>46019</v>
       </c>
     </row>

</xml_diff>